<commit_message>
Added Chapter 3 Vocabulary
</commit_message>
<xml_diff>
--- a/worksheets/Practice Worksheets.xlsx
+++ b/worksheets/Practice Worksheets.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schmu\source\repos\Greek\NT Greek FC-git\worksheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9778F3-4AF9-4795-BFF3-FF54D0BF6CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46A9916-409D-4AA4-BD3D-928CC0F21253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FC646E3-DDC1-46B0-B095-B13D94A96CEE}"/>
+    <workbookView xWindow="28755" yWindow="210" windowWidth="25395" windowHeight="15270" activeTab="1" xr2:uid="{4FC646E3-DDC1-46B0-B095-B13D94A96CEE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ch 2(a)" sheetId="1" r:id="rId1"/>
+    <sheet name="Ch 2" sheetId="1" r:id="rId1"/>
+    <sheet name="Ch 3 Masculine " sheetId="3" r:id="rId2"/>
+    <sheet name="Ch 3 Neuter" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Ch 2(a)'!$J$1:$T$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Ch 2'!$J$1:$T$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Ch 3 Masculine '!$J$1:$T$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Ch 3 Neuter'!$J$1:$T$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="7">
   <si>
     <t>Ch</t>
   </si>
@@ -125,9 +129,6 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -136,6 +137,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -419,6 +423,469 @@
         <a:xfrm>
           <a:off x="0" y="4238625"/>
           <a:ext cx="6050694" cy="3419475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF3B6FC1-73A4-4341-8C0A-450C60B40223}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6172200" y="2247900"/>
+          <a:ext cx="6696075" cy="2124075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A6554FD0-BA0A-4400-B945-BA2D7DC89229}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6172200" y="4505325"/>
+          <a:ext cx="6696075" cy="2124075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D77A8D4F-5CFA-4A6C-8279-55936D210064}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6172200" y="6743700"/>
+          <a:ext cx="6696075" cy="2124075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>500668</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B929F324-1035-8986-DACA-1BF7AA283569}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect b="49335"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="5987068" cy="3629025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7C0698A-AE97-4D56-BEB2-D7B81B8CC0A4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6172200" y="2247900"/>
+          <a:ext cx="6696075" cy="2124075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB72625E-EE70-44E5-8D56-5B80523A98CD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6172200" y="4505325"/>
+          <a:ext cx="6696075" cy="2124075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E0A4461-700D-4F3A-B64E-B443C5B46F9C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6172200" y="6743700"/>
+          <a:ext cx="6696075" cy="2124075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>180974</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>39040</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>28574</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF14F9F8-03F1-915D-5117-B95DAD06E7B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="180974"/>
+          <a:ext cx="6211240" cy="3362325"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -762,50 +1229,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="10:20">
-      <c r="J1" s="3"/>
-      <c r="K1" s="2" t="s">
+      <c r="J1" s="2"/>
+      <c r="K1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2" t="s">
+      <c r="L1" s="5"/>
+      <c r="M1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="2"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="2" t="s">
+      <c r="N1" s="5"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2" t="s">
+      <c r="R1" s="5"/>
+      <c r="S1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="2"/>
+      <c r="T1" s="5"/>
     </row>
     <row r="2" spans="10:20" ht="40.5" customHeight="1">
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="P2" s="4" t="s">
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="P2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5"/>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
     </row>
     <row r="3" spans="10:20" ht="38.25" customHeight="1">
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="Q3" s="1"/>
@@ -814,14 +1281,14 @@
       <c r="T3" s="1"/>
     </row>
     <row r="4" spans="10:20" ht="33.75" customHeight="1">
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
-      <c r="P4" s="4" t="s">
+      <c r="P4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="Q4" s="1"/>
@@ -830,14 +1297,14 @@
       <c r="T4" s="1"/>
     </row>
     <row r="5" spans="10:20" ht="39.75" customHeight="1">
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
-      <c r="P5" s="4" t="s">
+      <c r="P5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="Q5" s="1"/>
@@ -865,4 +1332,241 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57B98B20-DF0D-4A13-95E8-F3E0B4D3294A}">
+  <dimension ref="J1:T32"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="11" max="11" width="5.5" customWidth="1"/>
+    <col min="12" max="12" width="11.25" customWidth="1"/>
+    <col min="13" max="13" width="5.375" customWidth="1"/>
+    <col min="14" max="14" width="10.75" customWidth="1"/>
+    <col min="15" max="15" width="3.75" customWidth="1"/>
+    <col min="17" max="17" width="5.5" customWidth="1"/>
+    <col min="18" max="18" width="10.75" customWidth="1"/>
+    <col min="19" max="19" width="5.125" customWidth="1"/>
+    <col min="20" max="20" width="11.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="10:20">
+      <c r="J1" s="2"/>
+      <c r="K1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="5"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="T1" s="5"/>
+    </row>
+    <row r="2" spans="10:20" ht="40.5" customHeight="1">
+      <c r="J2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="P2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+    </row>
+    <row r="3" spans="10:20" ht="38.25" customHeight="1">
+      <c r="J3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="P3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+    </row>
+    <row r="4" spans="10:20" ht="33.75" customHeight="1">
+      <c r="J4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="P4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+    </row>
+    <row r="5" spans="10:20" ht="39.75" customHeight="1">
+      <c r="J5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+    </row>
+    <row r="6" spans="10:20" ht="10.5" customHeight="1"/>
+    <row r="19" ht="6.75" customHeight="1"/>
+    <row r="31" ht="12.75" customHeight="1"/>
+    <row r="32" ht="6.75" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:T1"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="1" max="16383" man="1"/>
+  </rowBreaks>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE0764C4-7AB5-439D-8D1C-4DB28FE61578}">
+  <dimension ref="J1:T32"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="11" max="11" width="5.5" customWidth="1"/>
+    <col min="12" max="12" width="11.25" customWidth="1"/>
+    <col min="13" max="13" width="5.375" customWidth="1"/>
+    <col min="14" max="14" width="10.75" customWidth="1"/>
+    <col min="15" max="15" width="3.75" customWidth="1"/>
+    <col min="17" max="17" width="5.5" customWidth="1"/>
+    <col min="18" max="18" width="10.75" customWidth="1"/>
+    <col min="19" max="19" width="5.125" customWidth="1"/>
+    <col min="20" max="20" width="11.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="10:20">
+      <c r="J1" s="2"/>
+      <c r="K1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="5"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="T1" s="5"/>
+    </row>
+    <row r="2" spans="10:20" ht="40.5" customHeight="1">
+      <c r="J2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="P2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+    </row>
+    <row r="3" spans="10:20" ht="38.25" customHeight="1">
+      <c r="J3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="P3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+    </row>
+    <row r="4" spans="10:20" ht="33.75" customHeight="1">
+      <c r="J4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="P4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+    </row>
+    <row r="5" spans="10:20" ht="39.75" customHeight="1">
+      <c r="J5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="P5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+    </row>
+    <row r="6" spans="10:20" ht="10.5" customHeight="1"/>
+    <row r="19" ht="6.75" customHeight="1"/>
+    <row r="31" ht="12.75" customHeight="1"/>
+    <row r="32" ht="6.75" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:T1"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>